<commit_message>
docs: implement senior feedback on F1 reports and README
</commit_message>
<xml_diff>
--- a/output/TMLT/LLM_Evaluation_Report.xlsx
+++ b/output/TMLT/LLM_Evaluation_Report.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Evaluation_Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Metrics_Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Data_Dictionary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:F201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,12 +448,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>System_Matched</t>
+          <t>AI_Prediction_is_Mapped</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>LLM_Agreed</t>
+          <t>Expert_Review_Agrees</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Evaluation_Result</t>
         </is>
       </c>
     </row>
@@ -463,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -472,10 +479,15 @@
         </is>
       </c>
       <c r="D2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -486,7 +498,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Eosinophils [+/-] in Stool by Light microscopy</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -495,10 +507,15 @@
         </is>
       </c>
       <c r="D3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -509,7 +526,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Gene panel testing for immunology (Trio analysis)</t>
+          <t>Pathology report</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -522,6 +539,11 @@
       </c>
       <c r="E4" t="b">
         <v>1</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -532,7 +554,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Phosphate [mg/dL] in Serum or Plasma</t>
+          <t>Phosphate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -545,6 +567,11 @@
       </c>
       <c r="E5" t="b">
         <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -555,7 +582,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Calcium [mg/dL] in Serum or Plasma</t>
+          <t>Calcium [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -568,6 +595,11 @@
       </c>
       <c r="E6" t="b">
         <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -578,7 +610,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Thyrotropin receptor Ab [U/mL] in Serum</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -587,10 +619,15 @@
         </is>
       </c>
       <c r="D7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -615,6 +652,11 @@
       <c r="E8" t="b">
         <v>0</v>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -624,7 +666,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>INR in Blood by Coagulation assay</t>
+          <t>Coagulation tissue factor-induced.INR in Platelet poor plasma by Coagulation assay</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -637,6 +679,11 @@
       </c>
       <c r="E9" t="b">
         <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -661,6 +708,11 @@
       <c r="E10" t="b">
         <v>1</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -670,7 +722,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Thyrotropin [mmol/L] in Serum or Plasma</t>
+          <t>Thyrotropin [Units/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -683,6 +735,11 @@
       </c>
       <c r="E11" t="b">
         <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -693,7 +750,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Bacteria identified in Tissue by Culture</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -702,10 +759,15 @@
         </is>
       </c>
       <c r="D12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -716,7 +778,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lambda light chains.free [mg/mL] in Serum by Nephelometry</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -725,10 +787,15 @@
         </is>
       </c>
       <c r="D13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -739,7 +806,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Calcium [mg/dL] in Urine</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -748,10 +815,15 @@
         </is>
       </c>
       <c r="D14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -776,6 +848,11 @@
       <c r="E15" t="b">
         <v>0</v>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -785,7 +862,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Protein/Creatinine [g/mmol cr] in Urine</t>
+          <t>Protein/Creatinine [Mass Ratio] in Urine</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -798,6 +875,11 @@
       </c>
       <c r="E16" t="b">
         <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -808,7 +890,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Phosphate [mg/dL] in Serum or Plasma</t>
+          <t>Phosphate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -821,6 +903,11 @@
       </c>
       <c r="E17" t="b">
         <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -831,7 +918,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Urinalysis panel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -840,10 +927,15 @@
         </is>
       </c>
       <c r="D18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -854,7 +946,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>INR in Blood by Coagulation assay</t>
+          <t>Coagulation tissue factor-induced.INR in Platelet poor plasma by Coagulation assay</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -867,6 +959,11 @@
       </c>
       <c r="E19" t="b">
         <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -877,7 +974,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -886,10 +983,15 @@
         </is>
       </c>
       <c r="D20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -914,6 +1016,11 @@
       <c r="E21" t="b">
         <v>0</v>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -923,7 +1030,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Phosphate [mg/dL] in Serum or Plasma</t>
+          <t>Phosphate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -936,6 +1043,11 @@
       </c>
       <c r="E22" t="b">
         <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -946,7 +1058,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Thyroxine (T4) free [ug/dL; ng/dL] in Serum or Plasma</t>
+          <t>Thyroxine.free [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -959,6 +1071,11 @@
       </c>
       <c r="E23" t="b">
         <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -969,7 +1086,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Phosphate [mg/dL] in Serum or Plasma</t>
+          <t>Phosphate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -982,6 +1099,11 @@
       </c>
       <c r="E24" t="b">
         <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1006,6 +1128,11 @@
       <c r="E25" t="b">
         <v>0</v>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1029,6 +1156,11 @@
       <c r="E26" t="b">
         <v>0</v>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1052,6 +1184,11 @@
       <c r="E27" t="b">
         <v>0</v>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1061,7 +1198,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Glucose tolerance panel in Serum or Plasma</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1070,10 +1207,15 @@
         </is>
       </c>
       <c r="D28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1098,6 +1240,11 @@
       <c r="E29" t="b">
         <v>0</v>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1107,7 +1254,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sodium [mmol/L] in Serum or Plasma</t>
+          <t>Sodium [Moles/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1120,6 +1267,11 @@
       </c>
       <c r="E30" t="b">
         <v>1</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1130,7 +1282,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Phosphate [mg/dL] in Serum or Plasma</t>
+          <t>Phosphate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1143,6 +1295,11 @@
       </c>
       <c r="E31" t="b">
         <v>1</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1153,7 +1310,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Paraneoplastic Ab Panel in Serum</t>
+          <t>Cyclic citrullinated peptide Ab [Units/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1165,7 +1322,12 @@
         <v>1</v>
       </c>
       <c r="E32" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>False Positive</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1176,7 +1338,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Clinical research drug XXX [ng/ml] in Urine</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1185,10 +1347,15 @@
         </is>
       </c>
       <c r="D33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1199,7 +1366,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pathology report</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1208,10 +1375,15 @@
         </is>
       </c>
       <c r="D34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1222,7 +1394,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1231,10 +1403,15 @@
         </is>
       </c>
       <c r="D35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1259,6 +1436,11 @@
       <c r="E36" t="b">
         <v>1</v>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1268,7 +1450,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mycobacterium sp DNA [+/-] in Serum or Plasma by NAA with probe detection</t>
+          <t>Mycobacterium tuberculosis complex DNA in Specimen by NAA with probe detection</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1281,6 +1463,11 @@
       </c>
       <c r="E37" t="b">
         <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1291,7 +1478,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yersinia sp identified in Stool by Organism specific culture</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1300,10 +1487,15 @@
         </is>
       </c>
       <c r="D38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E38" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1314,7 +1506,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Genetic screen in XXX specimen by Molecular genetics method Narrative</t>
+          <t>Chromosome analysis</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1327,6 +1519,11 @@
       </c>
       <c r="E39" t="b">
         <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1337,7 +1534,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Calcium [mg/dL] in Serum or Plasma</t>
+          <t>Calcium [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1350,6 +1547,11 @@
       </c>
       <c r="E40" t="b">
         <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1374,6 +1576,11 @@
       <c r="E41" t="b">
         <v>0</v>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1397,6 +1604,11 @@
       <c r="E42" t="b">
         <v>1</v>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>True Negative</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1406,7 +1618,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alkaline phosphatase [U/L] in Serum or Plasma</t>
+          <t>Alkaline phosphatase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1419,6 +1631,11 @@
       </c>
       <c r="E43" t="b">
         <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1429,7 +1646,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alkaline phosphatase [U/L] in Serum or Plasma</t>
+          <t>Alkaline phosphatase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1442,6 +1659,11 @@
       </c>
       <c r="E44" t="b">
         <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1452,7 +1674,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alkaline phosphatase [U/L] in Serum or Plasma</t>
+          <t>Alkaline phosphatase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1465,6 +1687,11 @@
       </c>
       <c r="E45" t="b">
         <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1475,7 +1702,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>activated Partial Thromboplatin Time aPTT in Platelet poor plasma by Coagulation assay</t>
+          <t>Coagulation surface induced [Time] in Platelet poor plasma by Coagulation assay</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1488,6 +1715,11 @@
       </c>
       <c r="E46" t="b">
         <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1512,6 +1744,11 @@
       <c r="E47" t="b">
         <v>1</v>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1521,7 +1758,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alkaline phosphatase [U/L] in Serum or Plasma</t>
+          <t>Alkaline phosphatase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1534,6 +1771,11 @@
       </c>
       <c r="E48" t="b">
         <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -1544,7 +1786,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Erythrocyte sedimentation rate [mm/hr] in Blood</t>
+          <t>Erythrocyte sedimentation rate</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1557,6 +1799,11 @@
       </c>
       <c r="E49" t="b">
         <v>1</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -1567,7 +1814,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Hemoglobin panel in Blood by Electrophoresis</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1576,10 +1823,15 @@
         </is>
       </c>
       <c r="D50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E50" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -1604,6 +1856,11 @@
       <c r="E51" t="b">
         <v>0</v>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1613,7 +1870,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Lactate [mmol/L] in Serum or Plasma</t>
+          <t>Lactate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1625,7 +1882,12 @@
         <v>1</v>
       </c>
       <c r="E52" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>False Positive</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -1650,6 +1912,11 @@
       <c r="E53" t="b">
         <v>1</v>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1659,7 +1926,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Microscopic observation [Identifier] in Tissue by Brown and Brenn stain</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1668,10 +1935,15 @@
         </is>
       </c>
       <c r="D54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E54" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -1682,7 +1954,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Skin biopsy (Dermatosis)</t>
+          <t>Pathology report</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1695,6 +1967,11 @@
       </c>
       <c r="E55" t="b">
         <v>1</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -1705,7 +1982,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Myelin oligodendrocyte glycoprotein Ab [Titer] in Serum by Cell binding immunofluorescent assay (CBA IFA)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1714,10 +1991,15 @@
         </is>
       </c>
       <c r="D56" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E56" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -1742,6 +2024,11 @@
       <c r="E57" t="b">
         <v>0</v>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1751,7 +2038,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ova and parasites identified in Stool by Parasite sedimentation</t>
+          <t>Parasite identified in Stool by Microscopy</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1764,6 +2051,11 @@
       </c>
       <c r="E58" t="b">
         <v>1</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -1774,7 +2066,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pathology report</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1783,10 +2075,15 @@
         </is>
       </c>
       <c r="D59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -1797,7 +2094,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>1,25-Dihydroxyvitamin D [pg/mL] in Serum or Plasma</t>
+          <t>25-hydroxycholecalciferol [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1810,6 +2107,11 @@
       </c>
       <c r="E60" t="b">
         <v>1</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -1820,7 +2122,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1829,10 +2131,15 @@
         </is>
       </c>
       <c r="D61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E61" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -1843,7 +2150,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Protein/Creatinine [g/mmol cr] in Urine</t>
+          <t>Protein/Creatinine [Mass Ratio] in Urine</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1856,6 +2163,11 @@
       </c>
       <c r="E62" t="b">
         <v>1</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -1880,6 +2192,11 @@
       <c r="E63" t="b">
         <v>1</v>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>True Negative</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1889,7 +2206,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Lactate dehydrogenase [U/L] in Synovial fluid by Lactate to pyruvate reaction</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1898,10 +2215,15 @@
         </is>
       </c>
       <c r="D64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E64" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -1912,7 +2234,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Thyroxine (T4) free [ug/dL; ng/dL] in Serum or Plasma</t>
+          <t>Thyroxine.free [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1925,6 +2247,11 @@
       </c>
       <c r="E65" t="b">
         <v>1</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -1935,7 +2262,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EGFR gene mutations tested for in Blood or Tissue by Molecular genetics method Nominal</t>
+          <t>Glomerular filtration rate/1.73 sq M.predicted [Volume Rate/Area] in Serum, Plasma or Blood by Creatinine-based formula (MDRD)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1948,6 +2275,11 @@
       </c>
       <c r="E66" t="b">
         <v>1</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -1958,7 +2290,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Cardiac Troponin I [ng/L] in Serum or Plasma by High sensitivity method</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1967,10 +2299,15 @@
         </is>
       </c>
       <c r="D67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E67" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -1995,6 +2332,11 @@
       <c r="E68" t="b">
         <v>1</v>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2004,7 +2346,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Prothrombin time (PT) [seconds]</t>
+          <t>Coagulation tissue factor-induced.time [Time] in Platelet poor plasma by Coagulation assay</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2017,6 +2359,11 @@
       </c>
       <c r="E69" t="b">
         <v>1</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -2041,6 +2388,11 @@
       <c r="E70" t="b">
         <v>0</v>
       </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2050,7 +2402,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Lipid profile (Cholesterol, HDL-chol,  LDL-chol, TG) in Serum or Plasma</t>
+          <t>Lipid panel in Serum or Plasma</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2063,6 +2415,11 @@
       </c>
       <c r="E71" t="b">
         <v>1</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -2073,7 +2430,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EGFR gene mutations tested for in Blood or Tissue by Molecular genetics method Nominal</t>
+          <t>Glomerular filtration rate/1.73 sq M.predicted [Volume Rate/Area] in Serum, Plasma or Blood by Creatinine-based formula (MDRD)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2086,6 +2443,11 @@
       </c>
       <c r="E72" t="b">
         <v>0</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>False Positive</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -2096,7 +2458,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Phosphate [mg/dL] in Serum or Plasma</t>
+          <t>Phosphate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2109,6 +2471,11 @@
       </c>
       <c r="E73" t="b">
         <v>1</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -2119,7 +2486,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Potassium [mmol/L] in Serum or Plasma</t>
+          <t>Potassium [Moles/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2132,6 +2499,11 @@
       </c>
       <c r="E74" t="b">
         <v>1</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -2142,7 +2514,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Microscopic observation [Identifier] in Tissue by Phosphotungstic acid Hematoxylin (PTAH) Stain</t>
+          <t>Pathology report</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2155,6 +2527,11 @@
       </c>
       <c r="E75" t="b">
         <v>1</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -2165,7 +2542,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Lactate [mmol/L] in Serum or Plasma</t>
+          <t>Lactate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2178,6 +2555,11 @@
       </c>
       <c r="E76" t="b">
         <v>1</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -2188,7 +2570,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Potassium [mmol/L] in Serum or Plasma</t>
+          <t>Potassium [Moles/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2201,6 +2583,11 @@
       </c>
       <c r="E77" t="b">
         <v>1</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -2211,7 +2598,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Erythrocyte sedimentation rate [mm/hr] in Blood</t>
+          <t>Erythrocyte sedimentation rate</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2224,6 +2611,11 @@
       </c>
       <c r="E78" t="b">
         <v>1</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -2234,7 +2626,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Parathyroid hormone Ag [+/-] in Tissue by Immune stain</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2243,10 +2635,15 @@
         </is>
       </c>
       <c r="D79" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E79" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -2271,6 +2668,11 @@
       <c r="E80" t="b">
         <v>1</v>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>True Negative</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2280,7 +2682,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Magnesium [mg/dL] in Serum or Plasma</t>
+          <t>Magnesium [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2293,6 +2695,11 @@
       </c>
       <c r="E81" t="b">
         <v>1</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -2317,6 +2724,11 @@
       <c r="E82" t="b">
         <v>1</v>
       </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2340,6 +2752,11 @@
       <c r="E83" t="b">
         <v>0</v>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2349,7 +2766,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Thyrotropin [mmol/L] in Serum or Plasma</t>
+          <t>Thyrotropin [Units/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2362,6 +2779,11 @@
       </c>
       <c r="E84" t="b">
         <v>1</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -2372,7 +2794,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Gamma glutamyl transferase [U/L] in Serum or Plasma</t>
+          <t>Gamma glutamyl transferase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2385,6 +2807,11 @@
       </c>
       <c r="E85" t="b">
         <v>1</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -2395,7 +2822,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Electrolytes panel in Urine</t>
+          <t>Electrolytes panel in Serum or Plasma</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2408,6 +2835,11 @@
       </c>
       <c r="E86" t="b">
         <v>1</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -2432,6 +2864,11 @@
       <c r="E87" t="b">
         <v>1</v>
       </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>True Negative</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2441,7 +2878,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Hemoglobin A1c/Hemoglobin.total [%] in Blood</t>
+          <t>Hemoglobin A1c/Hemoglobin.total in Blood</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2454,6 +2891,11 @@
       </c>
       <c r="E88" t="b">
         <v>1</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -2464,7 +2906,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EGFR gene mutations tested for in Blood or Tissue by Molecular genetics method Nominal</t>
+          <t>Glomerular filtration rate/1.73 sq M.predicted [Volume Rate/Area] in Serum, Plasma or Blood by Creatinine-based formula (MDRD)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2477,6 +2919,11 @@
       </c>
       <c r="E89" t="b">
         <v>1</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -2487,7 +2934,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Protein/Creatinine [g/mmol cr] in Urine</t>
+          <t>Protein/Creatinine [Mass Ratio] in Urine</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2500,6 +2947,11 @@
       </c>
       <c r="E90" t="b">
         <v>1</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -2524,6 +2976,11 @@
       <c r="E91" t="b">
         <v>0</v>
       </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2533,7 +2990,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Aspartate aminotransferase [U/L] in Serum or Plasma</t>
+          <t>Aspartate aminotransferase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2546,6 +3003,11 @@
       </c>
       <c r="E92" t="b">
         <v>0</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>False Positive</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -2570,6 +3032,11 @@
       <c r="E93" t="b">
         <v>1</v>
       </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2593,6 +3060,11 @@
       <c r="E94" t="b">
         <v>0</v>
       </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2602,7 +3074,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Bone Pathology biopsy report</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2611,10 +3083,15 @@
         </is>
       </c>
       <c r="D95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E95" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -2625,7 +3102,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Triiodothyronine (T3) Free [pmol/L] in Serum or Plasma by Immunoassay</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2634,10 +3111,15 @@
         </is>
       </c>
       <c r="D96" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E96" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -2648,7 +3130,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Interleukin 2 Receptor Soluble [pg/mL] in Serum or Plasma</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2657,10 +3139,15 @@
         </is>
       </c>
       <c r="D97" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E97" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -2671,7 +3158,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Creatinine [mg/dL] in Serum or Plasma</t>
+          <t>Creatinine [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2684,6 +3171,11 @@
       </c>
       <c r="E98" t="b">
         <v>1</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -2694,7 +3186,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Alkaline phosphatase [U/L] in Serum or Plasma</t>
+          <t>Alkaline phosphatase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2707,6 +3199,11 @@
       </c>
       <c r="E99" t="b">
         <v>1</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -2717,7 +3214,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Erythrocyte sedimentation rate [mm/hr] in Blood</t>
+          <t>Erythrocyte sedimentation rate</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2730,6 +3227,11 @@
       </c>
       <c r="E100" t="b">
         <v>1</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -2740,7 +3242,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Mycobacterium sp identified in Sputum by Organism specific culture</t>
+          <t>Mycobacterium sp identified in Specimen by Culture</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2753,6 +3255,11 @@
       </c>
       <c r="E101" t="b">
         <v>1</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -2763,7 +3270,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Erythrocyte sedimentation rate [mm/hr] in Blood</t>
+          <t>Erythrocyte sedimentation rate</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2776,6 +3283,11 @@
       </c>
       <c r="E102" t="b">
         <v>0</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>False Positive</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -2786,7 +3298,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Natural killer cell panel in Blood by Flow cytometry (FC)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2795,10 +3307,15 @@
         </is>
       </c>
       <c r="D103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E103" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -2809,7 +3326,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Parathion [ug/mL] in Serum or Plasma</t>
+          <t>Parathyrin.intact [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2822,6 +3339,11 @@
       </c>
       <c r="E104" t="b">
         <v>1</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -2832,7 +3354,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Gamma glutamyl transferase [U/L] in Serum or Plasma</t>
+          <t>Gamma glutamyl transferase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2845,6 +3367,11 @@
       </c>
       <c r="E105" t="b">
         <v>1</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -2869,6 +3396,11 @@
       <c r="E106" t="b">
         <v>1</v>
       </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2878,7 +3410,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Aldosterone/Renin [Ratio] in Plasma</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2887,10 +3419,15 @@
         </is>
       </c>
       <c r="D107" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E107" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="108">
@@ -2901,7 +3438,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Lead [mg/dL ; mcg/dL] in Serum or Plasma</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2910,10 +3447,15 @@
         </is>
       </c>
       <c r="D108" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E108" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -2938,6 +3480,11 @@
       <c r="E109" t="b">
         <v>1</v>
       </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>True Negative</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2947,7 +3494,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Calcium [mg/dL] in Serum or Plasma</t>
+          <t>Calcium [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2960,6 +3507,11 @@
       </c>
       <c r="E110" t="b">
         <v>1</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -2970,7 +3522,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>C reactive protein [mg/L] in Serum or Plasma</t>
+          <t>C reactive protein [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2983,6 +3535,11 @@
       </c>
       <c r="E111" t="b">
         <v>1</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="112">
@@ -2993,7 +3550,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Ketones [+/-] in Serum or Plasma</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3002,10 +3559,15 @@
         </is>
       </c>
       <c r="D112" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E112" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="113">
@@ -3016,7 +3578,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Erythrocyte sedimentation rate [mm/hr] in Blood</t>
+          <t>Erythrocyte sedimentation rate</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3029,6 +3591,11 @@
       </c>
       <c r="E113" t="b">
         <v>1</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -3053,6 +3620,11 @@
       <c r="E114" t="b">
         <v>1</v>
       </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3062,7 +3634,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Kidney needle biopsy (with immunohistochemical study)</t>
+          <t>Pathology report</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3075,6 +3647,11 @@
       </c>
       <c r="E115" t="b">
         <v>1</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="116">
@@ -3099,6 +3676,11 @@
       <c r="E116" t="b">
         <v>0</v>
       </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3108,7 +3690,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Creatinine [mg/dL] in Serum or Plasma</t>
+          <t>Creatinine [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3121,6 +3703,11 @@
       </c>
       <c r="E117" t="b">
         <v>1</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -3131,7 +3718,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3140,10 +3727,15 @@
         </is>
       </c>
       <c r="D118" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E118" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -3154,7 +3746,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Thyrotropin [mmol/L] in Serum or Plasma</t>
+          <t>Thyrotropin [Units/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3167,6 +3759,11 @@
       </c>
       <c r="E119" t="b">
         <v>1</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -3177,7 +3774,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Fungus identified in Synovial fluid by Culture</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3186,10 +3783,15 @@
         </is>
       </c>
       <c r="D120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E120" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -3200,7 +3802,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Thyroxine (T4) free [ug/dL; ng/dL] in Serum or Plasma</t>
+          <t>Thyroxine.free [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3213,6 +3815,11 @@
       </c>
       <c r="E121" t="b">
         <v>1</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -3223,7 +3830,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Synovial lining cells/cells [%] in Synovial fluid</t>
+          <t>Crystal identification in Synovial fluid by Microscopy</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3235,7 +3842,12 @@
         <v>1</v>
       </c>
       <c r="E122" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="123">
@@ -3246,7 +3858,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Parathion [ug/mL] in Serum or Plasma</t>
+          <t>Parathyrin.intact [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3259,6 +3871,11 @@
       </c>
       <c r="E123" t="b">
         <v>1</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -3269,7 +3886,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Creatinine [mg/dL] in Serum or Plasma</t>
+          <t>Creatinine [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3282,6 +3899,11 @@
       </c>
       <c r="E124" t="b">
         <v>1</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="125">
@@ -3292,7 +3914,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Creatinine [mg/dL] in Serum or Plasma</t>
+          <t>Creatinine [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3305,6 +3927,11 @@
       </c>
       <c r="E125" t="b">
         <v>1</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="126">
@@ -3315,7 +3942,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Thyroxine (T4) free [ug/dL; ng/dL] in Serum or Plasma</t>
+          <t>Thyroxine.free [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3328,6 +3955,11 @@
       </c>
       <c r="E126" t="b">
         <v>1</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -3338,7 +3970,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>EGFR gene mutations tested for in Blood or Tissue by Molecular genetics method Nominal</t>
+          <t>Glomerular filtration rate/1.73 sq M.predicted [Volume Rate/Area] in Serum, Plasma or Blood by Creatinine-based formula (MDRD)</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3351,6 +3983,11 @@
       </c>
       <c r="E127" t="b">
         <v>1</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="128">
@@ -3361,7 +3998,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Prothrombin time (PT) [seconds]</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3370,10 +4007,15 @@
         </is>
       </c>
       <c r="D128" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E128" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="129">
@@ -3384,7 +4026,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Plateletcrit [%] in Blood</t>
+          <t>Platelets [#/volume] in Blood by Automated count</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3397,6 +4039,11 @@
       </c>
       <c r="E129" t="b">
         <v>1</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="130">
@@ -3407,7 +4054,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pathology report</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3416,10 +4063,15 @@
         </is>
       </c>
       <c r="D130" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E130" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="131">
@@ -3430,7 +4082,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Paraneoplastic Ab Panel in Serum</t>
+          <t>Cyclic citrullinated peptide Ab [Units/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3443,6 +4095,11 @@
       </c>
       <c r="E131" t="b">
         <v>1</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="132">
@@ -3453,7 +4110,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Urine sediment comments by Light microscopy Narrative</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3462,10 +4119,15 @@
         </is>
       </c>
       <c r="D132" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E132" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="133">
@@ -3476,7 +4138,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Chromosome region 22q11.2 deletion and duplication mutation analysis (Digorge syndrome) in Blood or Tissue by FISH</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3485,10 +4147,15 @@
         </is>
       </c>
       <c r="D133" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E133" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="134">
@@ -3499,7 +4166,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Treponema pallidum Ab [Titer] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3508,10 +4175,15 @@
         </is>
       </c>
       <c r="D134" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E134" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="135">
@@ -3522,7 +4194,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Creatinine [mg/dL] in Serum or Plasma</t>
+          <t>Creatinine [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3535,6 +4207,11 @@
       </c>
       <c r="E135" t="b">
         <v>1</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -3545,7 +4222,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Synovial lining cells/cells [%] in Synovial fluid</t>
+          <t>Crystal identification in Synovial fluid by Microscopy</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3558,6 +4235,11 @@
       </c>
       <c r="E136" t="b">
         <v>1</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="137">
@@ -3568,7 +4250,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>C reactive protein [mg/L] in Serum or Plasma</t>
+          <t>C reactive protein [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3581,6 +4263,11 @@
       </c>
       <c r="E137" t="b">
         <v>1</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="138">
@@ -3591,7 +4278,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Microscopic observation [Identifier] in Tissue by Phosphotungstic acid Hematoxylin (PTAH) Stain</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3600,10 +4287,15 @@
         </is>
       </c>
       <c r="D138" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E138" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="139">
@@ -3614,7 +4306,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Parathyroid hormone Ag [+/-] in Tissue by Immune stain</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3623,10 +4315,15 @@
         </is>
       </c>
       <c r="D139" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E139" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="140">
@@ -3637,7 +4334,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Erythrocyte sedimentation rate [mm/hr] in Blood</t>
+          <t>Erythrocyte sedimentation rate</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3650,6 +4347,11 @@
       </c>
       <c r="E140" t="b">
         <v>1</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="141">
@@ -3660,7 +4362,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Lactate [mmol/L] in Serum or Plasma</t>
+          <t>Lactate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3673,6 +4375,11 @@
       </c>
       <c r="E141" t="b">
         <v>1</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="142">
@@ -3683,7 +4390,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Phosphate [mg/dL] in Serum or Plasma</t>
+          <t>Phosphate [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3696,6 +4403,11 @@
       </c>
       <c r="E142" t="b">
         <v>1</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="143">
@@ -3706,7 +4418,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Reticulocytes [10*9/L; 10*3/uL] in Blood</t>
+          <t>Reticulocytes [#/volume] in Blood</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3719,6 +4431,11 @@
       </c>
       <c r="E143" t="b">
         <v>1</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="144">
@@ -3729,7 +4446,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>activated Partial Thromboplatin Time aPTT in Platelet poor plasma by Coagulation assay</t>
+          <t>Coagulation surface induced [Time] in Platelet poor plasma by Coagulation assay</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3742,6 +4459,11 @@
       </c>
       <c r="E144" t="b">
         <v>1</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="145">
@@ -3752,7 +4474,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Mucopolysaccharides.microscopic observation [Identifier] in Tissue by Colloidal ferric oxide stain.Hale</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3761,10 +4483,15 @@
         </is>
       </c>
       <c r="D145" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E145" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="146">
@@ -3775,7 +4502,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pathology report</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3784,10 +4511,15 @@
         </is>
       </c>
       <c r="D146" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E146" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="147">
@@ -3798,7 +4530,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EGFR gene mutations tested for in Blood or Tissue by Molecular genetics method Nominal</t>
+          <t>Glomerular filtration rate/1.73 sq M.predicted [Volume Rate/Area] in Serum, Plasma or Blood by Creatinine-based formula (MDRD)</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3811,6 +4543,11 @@
       </c>
       <c r="E147" t="b">
         <v>1</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="148">
@@ -3821,7 +4558,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Ferritin [ng/mL] in Serum or Plasma by Immunoassay</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -3830,10 +4567,15 @@
         </is>
       </c>
       <c r="D148" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E148" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="149">
@@ -3844,7 +4586,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Electrolytes panel in Urine</t>
+          <t>Electrolytes panel in Serum or Plasma</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -3857,6 +4599,11 @@
       </c>
       <c r="E149" t="b">
         <v>1</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="150">
@@ -3881,6 +4628,11 @@
       <c r="E150" t="b">
         <v>0</v>
       </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3904,6 +4656,11 @@
       <c r="E151" t="b">
         <v>0</v>
       </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3913,7 +4670,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Plateletcrit [%] in Blood</t>
+          <t>Platelets [#/volume] in Blood by Automated count</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -3926,6 +4683,11 @@
       </c>
       <c r="E152" t="b">
         <v>1</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="153">
@@ -3936,7 +4698,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Hemoglobin [g/dL] in Blood</t>
+          <t>Hemoglobin [Mass/volume] in Blood</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -3949,6 +4711,11 @@
       </c>
       <c r="E153" t="b">
         <v>1</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="154">
@@ -3959,7 +4726,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3968,10 +4735,15 @@
         </is>
       </c>
       <c r="D154" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E154" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="155">
@@ -3982,7 +4754,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Thyrotropin [mmol/L] in Serum or Plasma</t>
+          <t>Thyrotropin [Units/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3995,6 +4767,11 @@
       </c>
       <c r="E155" t="b">
         <v>1</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="156">
@@ -4019,6 +4796,11 @@
       <c r="E156" t="b">
         <v>1</v>
       </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4028,7 +4810,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4037,10 +4819,15 @@
         </is>
       </c>
       <c r="D157" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E157" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="158">
@@ -4051,7 +4838,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Prothrombin time (PT) [seconds]</t>
+          <t>Coagulation tissue factor-induced.time [Time] in Platelet poor plasma by Coagulation assay</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4064,6 +4851,11 @@
       </c>
       <c r="E158" t="b">
         <v>1</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="159">
@@ -4074,7 +4866,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Centromere Ab [Titer] in Serum</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -4083,10 +4875,15 @@
         </is>
       </c>
       <c r="D159" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E159" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="160">
@@ -4097,7 +4894,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Aspartate aminotransferase [U/L] in Serum or Plasma</t>
+          <t>Aspartate aminotransferase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4110,6 +4907,11 @@
       </c>
       <c r="E160" t="b">
         <v>1</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="161">
@@ -4120,7 +4922,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Glucose tolerance panel in Serum or Plasma</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4129,10 +4931,15 @@
         </is>
       </c>
       <c r="D161" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E161" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="162">
@@ -4157,6 +4964,11 @@
       <c r="E162" t="b">
         <v>0</v>
       </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>False Positive</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4166,7 +4978,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Mycobacterium sp DNA [+/-] in Serum or Plasma by NAA with probe detection</t>
+          <t>Mycobacterium tuberculosis complex DNA in Specimen by NAA with probe detection</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4179,6 +4991,11 @@
       </c>
       <c r="E163" t="b">
         <v>1</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="164">
@@ -4203,6 +5020,11 @@
       <c r="E164" t="b">
         <v>1</v>
       </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -4226,6 +5048,11 @@
       <c r="E165" t="b">
         <v>1</v>
       </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -4235,7 +5062,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4244,10 +5071,15 @@
         </is>
       </c>
       <c r="D166" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E166" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="167">
@@ -4258,7 +5090,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Cobalamin (Vitamin B12) [pg/mL] in Serum or Plasma</t>
+          <t>Cobalamin [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4271,6 +5103,11 @@
       </c>
       <c r="E167" t="b">
         <v>1</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="168">
@@ -4281,7 +5118,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Calcium [mg/dL] in Serum or Plasma</t>
+          <t>Calcium [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4294,6 +5131,11 @@
       </c>
       <c r="E168" t="b">
         <v>1</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="169">
@@ -4304,7 +5146,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Bacteria identified in Stool by Culture</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4313,10 +5155,15 @@
         </is>
       </c>
       <c r="D169" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E169" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="170">
@@ -4341,6 +5188,11 @@
       <c r="E170" t="b">
         <v>1</v>
       </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -4350,7 +5202,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Treponema pallidum Ab [Titer] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4359,10 +5211,15 @@
         </is>
       </c>
       <c r="D171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E171" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="172">
@@ -4373,7 +5230,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Erythrocyte sedimentation rate [mm/hr] in Blood</t>
+          <t>Erythrocyte sedimentation rate</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -4386,6 +5243,11 @@
       </c>
       <c r="E172" t="b">
         <v>0</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>False Positive</t>
+        </is>
       </c>
     </row>
     <row r="173">
@@ -4396,7 +5258,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Glucose tolerance panel in Serum or Plasma</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4405,10 +5267,15 @@
         </is>
       </c>
       <c r="D173" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E173" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="174">
@@ -4419,7 +5286,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Alkaline phosphatase [U/L] in Serum or Plasma</t>
+          <t>Alkaline phosphatase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4432,6 +5299,11 @@
       </c>
       <c r="E174" t="b">
         <v>1</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="175">
@@ -4442,7 +5314,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4451,10 +5323,15 @@
         </is>
       </c>
       <c r="D175" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E175" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="176">
@@ -4465,7 +5342,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Chromosome analysis in Blood or Tissue by Microarray</t>
+          <t>Chromosome analysis</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -4478,6 +5355,11 @@
       </c>
       <c r="E176" t="b">
         <v>1</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="177">
@@ -4488,7 +5370,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Fungus identified in Synovial fluid by Culture</t>
+          <t>Fungus identified in Specimen by Culture</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4501,6 +5383,11 @@
       </c>
       <c r="E177" t="b">
         <v>1</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="178">
@@ -4511,7 +5398,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Creatinine [mg/dL] in Serum or Plasma</t>
+          <t>Creatinine [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -4524,6 +5411,11 @@
       </c>
       <c r="E178" t="b">
         <v>1</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="179">
@@ -4534,7 +5426,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Microscopic observation [Identifier] in Blood or Marrow by Sudan black B stain</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4543,10 +5435,15 @@
         </is>
       </c>
       <c r="D179" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E179" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="180">
@@ -4557,7 +5454,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Plateletcrit [%] in Blood</t>
+          <t>Platelets [#/volume] in Blood by Automated count</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4570,6 +5467,11 @@
       </c>
       <c r="E180" t="b">
         <v>1</v>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="181">
@@ -4580,7 +5482,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Hemoglobin [g/dL] in Blood</t>
+          <t>Hemoglobin [Mass/volume] in Blood</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4593,6 +5495,11 @@
       </c>
       <c r="E181" t="b">
         <v>1</v>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="182">
@@ -4603,7 +5510,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Cyclin D1 gene rearrangements [+/-] in Tissue by FISH</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4612,10 +5519,15 @@
         </is>
       </c>
       <c r="D182" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E182" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="183">
@@ -4626,7 +5538,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Microscopic observation [Identifier] in Blood or Marrow by Sudan black B stain</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4635,10 +5547,15 @@
         </is>
       </c>
       <c r="D183" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E183" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="184">
@@ -4649,7 +5566,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Parathion [ug/mL] in Serum or Plasma</t>
+          <t>Parathyrin.intact [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4662,6 +5579,11 @@
       </c>
       <c r="E184" t="b">
         <v>1</v>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="185">
@@ -4672,7 +5594,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Calcium [mg/dL] in Serum or Plasma</t>
+          <t>Calcium [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4685,6 +5607,11 @@
       </c>
       <c r="E185" t="b">
         <v>1</v>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="186">
@@ -4695,7 +5622,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Parathion [ug/mL] in Serum or Plasma</t>
+          <t>Parathyrin.intact [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -4708,6 +5635,11 @@
       </c>
       <c r="E186" t="b">
         <v>1</v>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="187">
@@ -4718,7 +5650,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Blood Gas Analysis panel (Blood)</t>
+          <t>Blood gas panel in Arterial blood</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -4731,6 +5663,11 @@
       </c>
       <c r="E187" t="b">
         <v>1</v>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="188">
@@ -4755,6 +5692,11 @@
       <c r="E188" t="b">
         <v>0</v>
       </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -4764,7 +5706,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Parathion [ug/mL] in Serum or Plasma</t>
+          <t>Parathyrin.intact [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -4777,6 +5719,11 @@
       </c>
       <c r="E189" t="b">
         <v>1</v>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="190">
@@ -4801,6 +5748,11 @@
       <c r="E190" t="b">
         <v>1</v>
       </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>True Negative</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4824,6 +5776,11 @@
       <c r="E191" t="b">
         <v>0</v>
       </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4833,7 +5790,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Creatinine [mg/dL] in Serum or Plasma</t>
+          <t>Creatinine [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -4846,6 +5803,11 @@
       </c>
       <c r="E192" t="b">
         <v>1</v>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="193">
@@ -4856,7 +5818,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Ethanol [mg/dL] in Serum or Plasma</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -4865,10 +5827,15 @@
         </is>
       </c>
       <c r="D193" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E193" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="194">
@@ -4879,7 +5846,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Alkaline phosphatase [U/L] in Serum or Plasma</t>
+          <t>Alkaline phosphatase [Enzymatic activity/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -4892,6 +5859,11 @@
       </c>
       <c r="E194" t="b">
         <v>1</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="195">
@@ -4916,6 +5888,11 @@
       <c r="E195" t="b">
         <v>1</v>
       </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -4939,6 +5916,11 @@
       <c r="E196" t="b">
         <v>1</v>
       </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>True Negative</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4948,7 +5930,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Hemoglobin A1c/Hemoglobin.total [%] in Blood</t>
+          <t>Hemoglobin A1c/Hemoglobin.total in Blood</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4961,6 +5943,11 @@
       </c>
       <c r="E197" t="b">
         <v>1</v>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="198">
@@ -4971,7 +5958,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Uterus with ovarian tumor</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -4980,10 +5967,15 @@
         </is>
       </c>
       <c r="D198" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E198" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
       </c>
     </row>
     <row r="199">
@@ -5008,6 +6000,11 @@
       <c r="E199" t="b">
         <v>0</v>
       </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>False Negative</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -5017,7 +6014,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Bilirubin.total [mg/dL ] in Serum or Plasma</t>
+          <t>Bilirubin.total [Mass/volume] in Serum or Plasma</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -5030,6 +6027,11 @@
       </c>
       <c r="E200" t="b">
         <v>1</v>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
       </c>
     </row>
     <row r="201">
@@ -5040,7 +6042,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Complete blood count in Blood by Automated count</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -5049,10 +6051,255 @@
         </is>
       </c>
       <c r="D201" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E201" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>True Positives (TP)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>132</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AI mapped correctly and Expert agreed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>False Positives (FP)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AI mapped it, but Expert says it is wrong (Hallucination)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>True Negatives (TN)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AI left it unmapped (-), and Expert agreed it should be unmapped</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>False Negatives (FN)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>54</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AI left it unmapped (-), but Expert says it could have been mapped</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.9496</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Accuracy of positive predictions (TP / (TP + FP))</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.7097</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ability to find all valid mappings (TP / (TP + FN))</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F1-Score</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.8123</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Harmonic mean of Precision and Recall</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Column Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lab_Item</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ชื่อรายการสั่งตรวจทางห้องปฏิบัติการจากฐานข้อมูล ICD-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TMLT_Name</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ชื่อมาตรฐาน TMLT ที่ระบบ AI ทำนายออกมา</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AI_Label</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ระดับความมั่นใจของ AI (Very High, High, Medium, Low, Rejected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AI_Prediction_is_Mapped</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ระบบ AI ได้ทำการจับคู่รหัสหรือไม่ (True = จับคู่, False = ปล่อยว่าง/Unmapped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Expert_Review_Agrees</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ผู้เชี่ยวชาญ (หรือ LLM Validator) เห็นด้วยกับการตัดสินใจของ AI หรือไม่</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Evaluation_Result</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ผลการประเมินทางสถิติ (True Positive, False Positive, True Negative, False Negative)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>